<commit_message>
Add seminar overview sheet to xlsx
Includes the target audience, lecturer, and main content header block
from the markdown source as a dedicated first sheet.
</commit_message>
<xml_diff>
--- a/enterprise_conquest_seminar.xlsx
+++ b/enterprise_conquest_seminar.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="スライド一覧" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="上司レビュー想定箇所" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="引用元一覧" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="セミナー概要" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="スライド一覧" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="上司レビュー想定箇所" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="引用元一覧" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -453,6 +454,72 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>項目</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>内容</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>対象セミナー</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>大手企業攻略に課題を持つマーケ・営業担当／責任者、新規事業責任者、スタートアップ・ベンチャー経営者向け</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>講師</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>名生 和史（株式会社BtoB AI Workers 代表）</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>メインコンテンツ</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>SIGQ社支援事例 deep dive（S11〜S22／12枚）</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1656,7 +1723,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1734,7 +1801,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>